<commit_message>
Support 'rebates included' flag per quote; skip rebate deductions when already net
</commit_message>
<xml_diff>
--- a/solar_battery_quotes.xlsx
+++ b/solar_battery_quotes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanking/Python/solar_analysis_output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1625356-C921-194D-8391-06C1B6940AAF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A60327-0353-CC40-B427-76CD66D47AB1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="3000" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{227D5E32-0A0C-8146-A00C-FA4E6E768303}"/>
+    <workbookView xWindow="5180" yWindow="3000" windowWidth="28040" windowHeight="17440" xr2:uid="{227D5E32-0A0C-8146-A00C-FA4E6E768303}"/>
   </bookViews>
   <sheets>
     <sheet name="quotes" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
   <si>
     <t>Quote number</t>
   </si>
@@ -47,13 +47,28 @@
   </si>
   <si>
     <t>PosEnergy</t>
+  </si>
+  <si>
+    <t>Plico</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes </t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Quote includes rebates?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,6 +80,22 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -90,9 +121,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -534,15 +567,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6332FF-2FEF-2A41-B284-2FB14DCDBE62}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="21.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.1640625" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="2" max="3" width="21.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.1640625" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -550,80 +583,197 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2">
         <v>33805</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <f>28*440/1000</f>
         <v>12.32</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>17.5</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3">
         <v>33875</v>
       </c>
-      <c r="D3">
-        <f t="shared" ref="D3:D4" si="0">15*440/1000</f>
+      <c r="E3">
+        <f t="shared" ref="E3:E4" si="0">15*440/1000</f>
         <v>6.6</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>26.3</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4">
         <v>28522</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <f t="shared" si="0"/>
         <v>6.6</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>17.5</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>10</v>
       </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>9988</v>
+      </c>
+      <c r="E5">
+        <v>6.6</v>
+      </c>
+      <c r="F5">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>13392</v>
+      </c>
+      <c r="E6">
+        <v>8.08</v>
+      </c>
+      <c r="F6">
+        <v>18.600000000000001</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>17928</v>
+      </c>
+      <c r="E7">
+        <v>9.9</v>
+      </c>
+      <c r="F7">
+        <v>27.9</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J15" s="3"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J16" s="3"/>
+    </row>
+    <row r="17" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J18" s="3"/>
+    </row>
+    <row r="19" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J20" s="3"/>
+    </row>
+    <row r="21" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J22" s="3"/>
+    </row>
+    <row r="23" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J23" s="3"/>
+    </row>
+    <row r="24" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J24" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update solar battery quotes spreadsheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solar_battery_quotes.xlsx
+++ b/solar_battery_quotes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanking/Python/solar_analysis_output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A60327-0353-CC40-B427-76CD66D47AB1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A9D5DD1-8DA6-CC45-84E9-4B443AD605D9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="3000" windowWidth="28040" windowHeight="17440" xr2:uid="{227D5E32-0A0C-8146-A00C-FA4E6E768303}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t>Quote number</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t xml:space="preserve">Yes </t>
-  </si>
-  <si>
-    <t>Yes</t>
   </si>
   <si>
     <t>Quote includes rebates?</t>
@@ -583,7 +580,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -681,62 +678,16 @@
         <v>9</v>
       </c>
       <c r="D5">
-        <v>9988</v>
+        <v>19720</v>
       </c>
       <c r="E5">
-        <v>6.6</v>
+        <v>15.675000000000001</v>
       </c>
       <c r="F5">
-        <v>9.3000000000000007</v>
+        <v>18.079999999999998</v>
       </c>
       <c r="G5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
         <v>10</v>
-      </c>
-      <c r="D6">
-        <v>13392</v>
-      </c>
-      <c r="E6">
-        <v>8.08</v>
-      </c>
-      <c r="F6">
-        <v>18.600000000000001</v>
-      </c>
-      <c r="G6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7">
-        <v>17928</v>
-      </c>
-      <c r="E7">
-        <v>9.9</v>
-      </c>
-      <c r="F7">
-        <v>27.9</v>
-      </c>
-      <c r="G7">
-        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update solar battery quotes spreadsheet and app
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solar_battery_quotes.xlsx
+++ b/solar_battery_quotes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanking/Python/solar_analysis_output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87219FB2-07D9-E242-B457-B891B2709E98}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EC2198A-A3D3-D64F-9823-FCD22AF18FD1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="3000" windowWidth="28040" windowHeight="17440" xr2:uid="{227D5E32-0A0C-8146-A00C-FA4E6E768303}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
   <si>
     <t>Quote number</t>
   </si>
@@ -145,15 +145,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>647700</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:colOff>635000</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>139700</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>138900</xdr:rowOff>
+      <xdr:colOff>127000</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>177000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -183,8 +183,69 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="9512300" y="927100"/>
+          <a:off x="9499600" y="3606800"/>
           <a:ext cx="7747000" cy="6527000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>444500</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="&lt;image001.png@01DCEDEE.EB83B930&gt;" descr="image001.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BEB1C25F-76D9-034F-8E58-E7B6017B37B7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9309100" y="368300"/>
+          <a:ext cx="9652000" cy="2705100"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -691,7 +752,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6332FF-2FEF-2A41-B284-2FB14DCDBE62}">
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="21.83203125" customWidth="1"/>
@@ -756,13 +817,13 @@
         <v>8</v>
       </c>
       <c r="D3">
-        <v>31388</v>
+        <v>32687</v>
       </c>
       <c r="E3">
-        <v>9.1999999999999993</v>
+        <v>13.8</v>
       </c>
       <c r="F3">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G3">
         <v>10</v>
@@ -779,13 +840,13 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>35270</v>
+        <v>31388</v>
       </c>
       <c r="E4">
         <v>9.1999999999999993</v>
       </c>
       <c r="F4">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G4">
         <v>10</v>
@@ -796,30 +857,49 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5">
-        <f>19720+1500</f>
-        <v>21220</v>
+        <v>35270</v>
       </c>
       <c r="E5">
-        <v>15.675000000000001</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="F5">
-        <v>18.079999999999998</v>
+        <v>36</v>
       </c>
       <c r="G5">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J13" s="2"/>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6">
+        <v>21220</v>
+      </c>
+      <c r="E6">
+        <v>15.675000000000001</v>
+      </c>
+      <c r="F6">
+        <v>18.079999999999998</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J14" s="3"/>
+      <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J15" s="3"/>
@@ -828,10 +908,10 @@
       <c r="J16" s="3"/>
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.2">
-      <c r="J17" s="2"/>
+      <c r="J17" s="3"/>
     </row>
     <row r="18" spans="10:10" x14ac:dyDescent="0.2">
-      <c r="J18" s="3"/>
+      <c r="J18" s="2"/>
     </row>
     <row r="19" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J19" s="3"/>
@@ -840,16 +920,19 @@
       <c r="J20" s="3"/>
     </row>
     <row r="21" spans="10:10" x14ac:dyDescent="0.2">
-      <c r="J21" s="2"/>
+      <c r="J21" s="3"/>
     </row>
     <row r="22" spans="10:10" x14ac:dyDescent="0.2">
-      <c r="J22" s="3"/>
+      <c r="J22" s="2"/>
     </row>
     <row r="23" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J23" s="3"/>
     </row>
     <row r="24" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J24" s="3"/>
+    </row>
+    <row r="25" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J25" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update solar battery quotes spreadsheet (corrected)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solar_battery_quotes.xlsx
+++ b/solar_battery_quotes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanking/Python/solar_analysis_output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97CF9607-9B8D-CE4F-8227-5D8034E35275}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C60462B1-48AB-B040-844E-87DA2287CD5E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="3000" windowWidth="28040" windowHeight="17440" xr2:uid="{227D5E32-0A0C-8146-A00C-FA4E6E768303}"/>
   </bookViews>
@@ -53,10 +53,10 @@
     <t>Quote includes rebates?</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
+    <t>Vendor A</t>
+  </si>
+  <si>
+    <t>Vendor B</t>
   </si>
 </sst>
 </file>
@@ -142,255 +142,6 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>596900</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>88900</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>24600</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="&lt;image004.png@01DCEDDC.8E8FF7A0&gt;" descr="image004.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09FD0F64-2451-6A4B-9459-AEA2DA1F4706}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="9461500" y="3657600"/>
-          <a:ext cx="7747000" cy="6527000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>444500</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="&lt;image001.png@01DCEDEE.EB83B930&gt;" descr="image001.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BEB1C25F-76D9-034F-8E58-E7B6017B37B7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="9309100" y="368300"/>
-          <a:ext cx="9652000" cy="2705100"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>698500</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="&lt;image008.png@01DCD988.70044560&gt;" descr="image008.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{61FDC39F-62A2-C043-A6EA-CA0EE3C7587C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="8255000" y="609600"/>
-          <a:ext cx="9779000" cy="2692400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>660400</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="&lt;image001.png@01DCE215.8B9CEC60&gt;" descr="image001.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A768B37-E478-8B4F-B887-62BF0F5FF3EC}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="7429500" y="5283200"/>
-          <a:ext cx="9740900" cy="5334000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
@@ -416,7 +167,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -446,6 +197,111 @@
             </a14:hiddenFill>
           </a:ext>
         </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>635000</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="&lt;image001.png@01DCEDEE.EB83B930&gt;" descr="image001.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4AADBC3E-C8DA-7848-B67D-B33E425B67DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8191500" y="508000"/>
+          <a:ext cx="8128000" cy="2273300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>790780</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>771992</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5335058F-2A67-2341-B0D1-D5ADB112B4E5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8220280" y="2971800"/>
+          <a:ext cx="8236212" cy="3479800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -934,7 +790,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add in-app quote editor and update quotes spreadsheet
- solar_battery_quotes.xlsx: updated with 4 current installer quotes
- solar_battery_analyser.py: load_quotes_from_file now returns per-quote
  shading 9-tuples; add_solar/solar_profile accept optional shade tuple;
  Excel output includes per-quote shading columns
- app.py: replace static quotes dropdown with editable data_editor table;
  add optional quotes file uploader; add download-as-Excel button so
  edited quotes can be committed back to git

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solar_battery_quotes.xlsx
+++ b/solar_battery_quotes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanking/Python/solar_analysis_output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{403D71A3-51E6-334A-A1EA-64367F626846}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8FFD8B-1359-204F-B515-580C8A357BAB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="3220" windowWidth="28040" windowHeight="17440" xr2:uid="{227D5E32-0A0C-8146-A00C-FA4E6E768303}"/>
+    <workbookView xWindow="4840" yWindow="5580" windowWidth="28040" windowHeight="17440" xr2:uid="{227D5E32-0A0C-8146-A00C-FA4E6E768303}"/>
   </bookViews>
   <sheets>
     <sheet name="quotes" sheetId="1" r:id="rId1"/>
@@ -740,7 +740,8 @@
         <v>6</v>
       </c>
       <c r="D3">
-        <v>19720</v>
+        <f>18736+1500+1088</f>
+        <v>21324</v>
       </c>
       <c r="E3">
         <v>15.675000000000001</v>

</xml_diff>

<commit_message>
Update solar battery pricing spreadsheet
</commit_message>
<xml_diff>
--- a/solar_battery_quotes.xlsx
+++ b/solar_battery_quotes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanking/Python/solar_analysis_output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8FFD8B-1359-204F-B515-580C8A357BAB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A04FFB2-7F92-5C40-9F39-0477DBF7CF8B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4840" yWindow="5580" windowWidth="28040" windowHeight="17440" xr2:uid="{227D5E32-0A0C-8146-A00C-FA4E6E768303}"/>
   </bookViews>
@@ -740,8 +740,7 @@
         <v>6</v>
       </c>
       <c r="D3">
-        <f>18736+1500+1088</f>
-        <v>21324</v>
+        <v>19824</v>
       </c>
       <c r="E3">
         <v>15.675000000000001</v>

</xml_diff>